<commit_message>
Bottom Board BOM updated #160
</commit_message>
<xml_diff>
--- a/Design-Files/SM_Bottom_Board_v3.3/BOM/eSpark-BOM-Bottom (20 Board).xlsx
+++ b/Design-Files/SM_Bottom_Board_v3.3/BOM/eSpark-BOM-Bottom (20 Board).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Deliverables\SM_Bottom Board\_BOM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Faizan\GitHub\ColeBenson-SmartMotors\Design-Files\SM_Bottom_Board_v3.3\BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80F0F123-5582-4C09-B5D2-11D3E2F71EF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{912DF0CD-7358-45BD-89BA-A5336B904C37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="214">
   <si>
     <t>Component list</t>
   </si>
@@ -77,9 +77,6 @@
     <t>C18, C19</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
     <t>D12</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>Rx1, Rx2</t>
   </si>
   <si>
-    <t>SB1, SB2, SB3, SB4, SB5, SB6, SB7, SB8</t>
-  </si>
-  <si>
     <t>SW1</t>
   </si>
   <si>
@@ -173,9 +167,6 @@
     <t>CAP CER 10PF 25V C0G 0201</t>
   </si>
   <si>
-    <t>TVS DIODE 24VWM 41VC TO236AB</t>
-  </si>
-  <si>
     <t>TVS DIODE 5V 9.8V SOD923</t>
   </si>
   <si>
@@ -218,9 +209,6 @@
     <t>RES SMD 100 OHM 1% 1/10W 0603</t>
   </si>
   <si>
-    <t>Solder Bridge ON</t>
-  </si>
-  <si>
     <t>No NO J pin 50mA 3mm 100MΩ 100000 12V 250gf@±30gf 2.6mm -30℃~+85℃ 0.65mm Black Round Button Brick nogging SPST SMD Tactile Switches ROHS</t>
   </si>
   <si>
@@ -290,9 +278,6 @@
     <t>Res0603</t>
   </si>
   <si>
-    <t>Solder Bridge</t>
-  </si>
-  <si>
     <t>GT-TC025D-H0065-L1</t>
   </si>
   <si>
@@ -335,9 +320,6 @@
     <t>CGA1A2C0G1E100D030BA</t>
   </si>
   <si>
-    <t>PESD2CAN,215</t>
-  </si>
-  <si>
     <t>ESD9L5.0ST5G</t>
   </si>
   <si>
@@ -410,9 +392,6 @@
     <t>TDK</t>
   </si>
   <si>
-    <t>Nexperia</t>
-  </si>
-  <si>
     <t>ON Semiconductor</t>
   </si>
   <si>
@@ -585,9 +564,6 @@
   </si>
   <si>
     <t>C2168858</t>
-  </si>
-  <si>
-    <t>C75176</t>
   </si>
   <si>
     <t>C82326</t>
@@ -710,7 +686,7 @@
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="27" x14ac:knownFonts="1">
+  <fonts count="25" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -865,23 +841,6 @@
     <font>
       <strike/>
       <sz val="9"/>
-      <color rgb="FFC00000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <strike/>
-      <sz val="9"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <strike/>
-      <sz val="9"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -1194,9 +1153,9 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1375,37 +1334,22 @@
     <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="24" fillId="2" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1417,9 +1361,6 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1441,7 +1382,7 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1474,7 +1415,7 @@
     <xf numFmtId="0" fontId="19" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="2" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1845,29 +1786,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:R43"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:R41"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
+    <col min="2" max="2" width="3.109375" style="26" customWidth="1"/>
     <col min="3" max="3" width="18" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="26.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.44140625" customWidth="1"/>
+    <col min="5" max="5" width="30.88671875" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="26.44140625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="8.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="8.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="26.88671875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="22.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -1878,16 +1820,16 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="100"/>
-      <c r="L1" s="100"/>
-      <c r="M1" s="100"/>
-      <c r="N1" s="100"/>
-      <c r="O1" s="100"/>
-      <c r="P1" s="100"/>
-      <c r="Q1" s="100"/>
-      <c r="R1" s="101"/>
-    </row>
-    <row r="2" spans="1:18" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="K1" s="94"/>
+      <c r="L1" s="94"/>
+      <c r="M1" s="94"/>
+      <c r="N1" s="94"/>
+      <c r="O1" s="94"/>
+      <c r="P1" s="94"/>
+      <c r="Q1" s="94"/>
+      <c r="R1" s="95"/>
+    </row>
+    <row r="2" spans="1:18" ht="31.8" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1"/>
       <c r="B2" s="21"/>
       <c r="C2" s="32"/>
@@ -1896,7 +1838,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="56" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="4"/>
@@ -1911,7 +1853,7 @@
       <c r="Q2" s="4"/>
       <c r="R2" s="3"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
       <c r="B3" s="22"/>
       <c r="C3" s="33"/>
@@ -1920,7 +1862,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="57" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="5"/>
@@ -1933,9 +1875,9 @@
       <c r="O3" s="5"/>
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
-      <c r="R3" s="102"/>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R3" s="96"/>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="22"/>
       <c r="C4" s="33"/>
@@ -1944,7 +1886,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="58" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="7"/>
@@ -1957,9 +1899,9 @@
       <c r="O4" s="6"/>
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
-      <c r="R4" s="103"/>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R4" s="97"/>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
       <c r="B5" s="22"/>
       <c r="C5" s="33"/>
@@ -1981,9 +1923,9 @@
       <c r="O5" s="6"/>
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
-      <c r="R5" s="103"/>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R5" s="97"/>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
       <c r="B6" s="23"/>
       <c r="C6" s="34"/>
@@ -2001,9 +1943,9 @@
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
-      <c r="R6" s="103"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R6" s="97"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
       <c r="B7" s="24"/>
       <c r="C7" s="35"/>
@@ -2021,9 +1963,9 @@
       <c r="O7" s="8"/>
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
-      <c r="R7" s="103"/>
-    </row>
-    <row r="8" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R7" s="97"/>
+    </row>
+    <row r="8" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8" s="1"/>
       <c r="B8" s="27"/>
       <c r="C8" s="36"/>
@@ -2041,1305 +1983,1308 @@
       <c r="O8" s="8"/>
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
-      <c r="R8" s="103"/>
-    </row>
-    <row r="9" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="R8" s="97"/>
+    </row>
+    <row r="9" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="1"/>
       <c r="B9" s="30" t="s">
         <v>4</v>
       </c>
       <c r="C9" s="30" t="s">
-        <v>156</v>
+        <v>149</v>
       </c>
       <c r="D9" s="30" t="s">
         <v>8</v>
       </c>
       <c r="E9" s="31" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="F9" s="61" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="G9" s="30" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="H9" s="60" t="s">
-        <v>119</v>
+        <v>113</v>
       </c>
       <c r="I9" s="30" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
       <c r="J9" s="30" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="K9" s="31" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="L9" s="30" t="s">
+        <v>148</v>
+      </c>
+      <c r="M9" s="30" t="s">
+        <v>151</v>
+      </c>
+      <c r="N9" s="60" t="s">
+        <v>152</v>
+      </c>
+      <c r="O9" s="30" t="s">
+        <v>153</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>154</v>
+      </c>
+      <c r="Q9" s="60" t="s">
         <v>155</v>
       </c>
-      <c r="M9" s="30" t="s">
-        <v>158</v>
-      </c>
-      <c r="N9" s="60" t="s">
-        <v>159</v>
-      </c>
-      <c r="O9" s="30" t="s">
-        <v>160</v>
-      </c>
-      <c r="P9" s="30" t="s">
-        <v>161</v>
-      </c>
-      <c r="Q9" s="60" t="s">
-        <v>162</v>
-      </c>
       <c r="R9" s="30" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
       <c r="B10" s="50">
         <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="92" t="s">
-        <v>164</v>
-      </c>
-      <c r="D10" s="93" t="s">
+      <c r="C10" s="86" t="s">
+        <v>157</v>
+      </c>
+      <c r="D10" s="87" t="s">
         <v>9</v>
       </c>
-      <c r="E10" s="93" t="s">
-        <v>40</v>
-      </c>
-      <c r="F10" s="94" t="s">
-        <v>73</v>
-      </c>
-      <c r="G10" s="93" t="s">
-        <v>94</v>
-      </c>
-      <c r="H10" s="94" t="s">
-        <v>120</v>
-      </c>
-      <c r="I10" s="93" t="s">
-        <v>176</v>
-      </c>
-      <c r="J10" s="94" t="s">
-        <v>178</v>
-      </c>
-      <c r="K10" s="93" t="s">
-        <v>142</v>
-      </c>
-      <c r="L10" s="95">
+      <c r="E10" s="87" t="s">
+        <v>38</v>
+      </c>
+      <c r="F10" s="88" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" s="88" t="s">
+        <v>114</v>
+      </c>
+      <c r="I10" s="87" t="s">
+        <v>169</v>
+      </c>
+      <c r="J10" s="88" t="s">
+        <v>171</v>
+      </c>
+      <c r="K10" s="87" t="s">
+        <v>135</v>
+      </c>
+      <c r="L10" s="89">
         <v>1</v>
       </c>
-      <c r="M10" s="93">
+      <c r="M10" s="87">
         <f>L10*20</f>
         <v>20</v>
       </c>
-      <c r="N10" s="94">
+      <c r="N10" s="88">
         <v>40</v>
       </c>
-      <c r="O10" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P10" s="96">
+      <c r="O10" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P10" s="90">
         <v>1.7399999999999999E-2</v>
       </c>
-      <c r="Q10" s="97">
+      <c r="Q10" s="91">
         <f>P10*N10</f>
         <v>0.69599999999999995</v>
       </c>
-      <c r="R10" s="98"/>
-    </row>
-    <row r="11" spans="1:18" ht="36" x14ac:dyDescent="0.25">
+      <c r="R10" s="92"/>
+    </row>
+    <row r="11" spans="1:18" ht="24" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="51">
-        <f t="shared" ref="B11:B40" si="0">ROW(B11) - ROW($B$9)</f>
+        <f t="shared" ref="B11:B38" si="0">ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
-      <c r="C11" s="85" t="s">
-        <v>164</v>
-      </c>
-      <c r="D11" s="86" t="s">
-        <v>217</v>
-      </c>
-      <c r="E11" s="86" t="s">
-        <v>41</v>
-      </c>
-      <c r="F11" s="87" t="s">
-        <v>73</v>
-      </c>
-      <c r="G11" s="86" t="s">
-        <v>95</v>
-      </c>
-      <c r="H11" s="87" t="s">
-        <v>120</v>
-      </c>
-      <c r="I11" s="86" t="s">
-        <v>176</v>
-      </c>
-      <c r="J11" s="87" t="s">
-        <v>179</v>
-      </c>
-      <c r="K11" s="86" t="s">
-        <v>143</v>
-      </c>
-      <c r="L11" s="89">
+      <c r="C11" s="79" t="s">
+        <v>157</v>
+      </c>
+      <c r="D11" s="80" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="80" t="s">
+        <v>39</v>
+      </c>
+      <c r="F11" s="81" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" s="80" t="s">
+        <v>90</v>
+      </c>
+      <c r="H11" s="81" t="s">
+        <v>114</v>
+      </c>
+      <c r="I11" s="80" t="s">
+        <v>169</v>
+      </c>
+      <c r="J11" s="81" t="s">
+        <v>172</v>
+      </c>
+      <c r="K11" s="80" t="s">
+        <v>136</v>
+      </c>
+      <c r="L11" s="83">
         <v>18</v>
       </c>
-      <c r="M11" s="86">
-        <f t="shared" ref="M11:M41" si="1">L11*20</f>
+      <c r="M11" s="80">
+        <f t="shared" ref="M11:M39" si="1">L11*20</f>
         <v>360</v>
       </c>
-      <c r="N11" s="87">
+      <c r="N11" s="81">
         <v>400</v>
       </c>
-      <c r="O11" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P11" s="90">
+      <c r="O11" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P11" s="84">
         <v>2.3999999999999998E-3</v>
       </c>
-      <c r="Q11" s="91">
+      <c r="Q11" s="85">
         <f t="shared" ref="Q11" si="2">P11*N11</f>
         <v>0.96</v>
       </c>
-      <c r="R11" s="86"/>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R11" s="80"/>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="50">
         <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
-      <c r="C12" s="92" t="s">
-        <v>164</v>
-      </c>
-      <c r="D12" s="93" t="s">
+      <c r="C12" s="86" t="s">
+        <v>157</v>
+      </c>
+      <c r="D12" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="E12" s="93" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="94" t="s">
-        <v>203</v>
-      </c>
-      <c r="G12" s="93" t="s">
-        <v>96</v>
-      </c>
-      <c r="H12" s="94" t="s">
-        <v>121</v>
-      </c>
-      <c r="I12" s="93" t="s">
-        <v>176</v>
-      </c>
-      <c r="J12" s="94" t="s">
-        <v>180</v>
-      </c>
-      <c r="K12" s="93" t="s">
-        <v>175</v>
-      </c>
-      <c r="L12" s="95">
+      <c r="E12" s="87" t="s">
+        <v>40</v>
+      </c>
+      <c r="F12" s="88" t="s">
+        <v>195</v>
+      </c>
+      <c r="G12" s="87" t="s">
+        <v>91</v>
+      </c>
+      <c r="H12" s="88" t="s">
+        <v>115</v>
+      </c>
+      <c r="I12" s="87" t="s">
+        <v>169</v>
+      </c>
+      <c r="J12" s="88" t="s">
+        <v>173</v>
+      </c>
+      <c r="K12" s="87" t="s">
+        <v>168</v>
+      </c>
+      <c r="L12" s="89">
         <v>1</v>
       </c>
-      <c r="M12" s="93">
+      <c r="M12" s="87">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N12" s="94">
+      <c r="N12" s="88">
         <v>25</v>
       </c>
-      <c r="O12" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P12" s="96">
+      <c r="O12" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P12" s="90">
         <v>5.2600000000000001E-2</v>
       </c>
-      <c r="Q12" s="97">
+      <c r="Q12" s="91">
         <f>P12*N12</f>
         <v>1.3149999999999999</v>
       </c>
-      <c r="R12" s="93"/>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R12" s="87"/>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
       <c r="B13" s="51">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="85" t="s">
-        <v>164</v>
-      </c>
-      <c r="D13" s="86" t="s">
+      <c r="C13" s="79" t="s">
+        <v>157</v>
+      </c>
+      <c r="D13" s="80" t="s">
         <v>11</v>
       </c>
-      <c r="E13" s="86" t="s">
-        <v>43</v>
-      </c>
-      <c r="F13" s="87" t="s">
-        <v>74</v>
-      </c>
-      <c r="G13" s="86" t="s">
-        <v>97</v>
-      </c>
-      <c r="H13" s="87" t="s">
-        <v>122</v>
-      </c>
-      <c r="I13" s="86" t="s">
-        <v>176</v>
-      </c>
-      <c r="J13" s="87" t="s">
-        <v>181</v>
-      </c>
-      <c r="K13" s="86" t="s">
-        <v>144</v>
-      </c>
-      <c r="L13" s="89">
+      <c r="E13" s="80" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="81" t="s">
+        <v>70</v>
+      </c>
+      <c r="G13" s="80" t="s">
+        <v>92</v>
+      </c>
+      <c r="H13" s="81" t="s">
+        <v>116</v>
+      </c>
+      <c r="I13" s="80" t="s">
+        <v>169</v>
+      </c>
+      <c r="J13" s="81" t="s">
+        <v>174</v>
+      </c>
+      <c r="K13" s="80" t="s">
+        <v>137</v>
+      </c>
+      <c r="L13" s="83">
         <v>2</v>
       </c>
-      <c r="M13" s="86">
+      <c r="M13" s="80">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N13" s="87">
+      <c r="N13" s="81">
         <v>50</v>
       </c>
-      <c r="O13" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P13" s="90">
+      <c r="O13" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P13" s="84">
         <v>5.96E-2</v>
       </c>
-      <c r="Q13" s="91">
+      <c r="Q13" s="85">
         <f t="shared" ref="Q13" si="3">P13*N13</f>
         <v>2.98</v>
       </c>
-      <c r="R13" s="86"/>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R13" s="80"/>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="50">
         <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
-      <c r="C14" s="92" t="s">
-        <v>164</v>
-      </c>
-      <c r="D14" s="93" t="s">
+      <c r="C14" s="86" t="s">
+        <v>157</v>
+      </c>
+      <c r="D14" s="87" t="s">
         <v>12</v>
       </c>
-      <c r="E14" s="93" t="s">
-        <v>44</v>
-      </c>
-      <c r="F14" s="94" t="s">
-        <v>74</v>
-      </c>
-      <c r="G14" s="93" t="s">
-        <v>98</v>
-      </c>
-      <c r="H14" s="94" t="s">
-        <v>123</v>
-      </c>
-      <c r="I14" s="93" t="s">
-        <v>176</v>
-      </c>
-      <c r="J14" s="94" t="s">
-        <v>182</v>
-      </c>
-      <c r="K14" s="93" t="s">
-        <v>145</v>
-      </c>
-      <c r="L14" s="95">
+      <c r="E14" s="87" t="s">
+        <v>42</v>
+      </c>
+      <c r="F14" s="88" t="s">
+        <v>70</v>
+      </c>
+      <c r="G14" s="87" t="s">
+        <v>93</v>
+      </c>
+      <c r="H14" s="88" t="s">
+        <v>117</v>
+      </c>
+      <c r="I14" s="87" t="s">
+        <v>169</v>
+      </c>
+      <c r="J14" s="88" t="s">
+        <v>175</v>
+      </c>
+      <c r="K14" s="87" t="s">
+        <v>138</v>
+      </c>
+      <c r="L14" s="89">
         <v>2</v>
       </c>
-      <c r="M14" s="93">
+      <c r="M14" s="87">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N14" s="94">
+      <c r="N14" s="88">
         <v>100</v>
       </c>
-      <c r="O14" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P14" s="96">
+      <c r="O14" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P14" s="90">
         <v>2.5999999999999999E-3</v>
       </c>
-      <c r="Q14" s="97">
+      <c r="Q14" s="91">
         <f>P14*N14</f>
         <v>0.26</v>
       </c>
-      <c r="R14" s="93"/>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R14" s="87"/>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="51">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="85" t="s">
-        <v>164</v>
-      </c>
-      <c r="D15" s="86" t="s">
+      <c r="C15" s="79" t="s">
+        <v>157</v>
+      </c>
+      <c r="D15" s="80" t="s">
         <v>13</v>
       </c>
-      <c r="E15" s="86" t="s">
-        <v>45</v>
-      </c>
-      <c r="F15" s="87" t="s">
-        <v>75</v>
-      </c>
-      <c r="G15" s="88" t="s">
-        <v>99</v>
-      </c>
-      <c r="H15" s="87" t="s">
-        <v>124</v>
-      </c>
-      <c r="I15" s="86" t="s">
-        <v>209</v>
-      </c>
-      <c r="J15" s="87" t="s">
-        <v>183</v>
-      </c>
-      <c r="K15" s="86" t="s">
-        <v>146</v>
-      </c>
-      <c r="L15" s="89">
+      <c r="E15" s="80" t="s">
+        <v>43</v>
+      </c>
+      <c r="F15" s="81" t="s">
+        <v>71</v>
+      </c>
+      <c r="G15" s="82" t="s">
+        <v>94</v>
+      </c>
+      <c r="H15" s="81" t="s">
+        <v>118</v>
+      </c>
+      <c r="I15" s="80" t="s">
+        <v>201</v>
+      </c>
+      <c r="J15" s="81" t="s">
+        <v>176</v>
+      </c>
+      <c r="K15" s="80" t="s">
+        <v>139</v>
+      </c>
+      <c r="L15" s="83">
         <v>2</v>
       </c>
-      <c r="M15" s="86">
+      <c r="M15" s="80">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N15" s="87">
+      <c r="N15" s="81">
         <v>50</v>
       </c>
-      <c r="O15" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P15" s="90">
+      <c r="O15" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P15" s="84">
         <v>6.4000000000000003E-3</v>
       </c>
-      <c r="Q15" s="91">
+      <c r="Q15" s="85">
         <f t="shared" ref="Q15" si="4">P15*N15</f>
         <v>0.32</v>
       </c>
-      <c r="R15" s="86"/>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R15" s="80"/>
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="51">
-        <f t="shared" si="0"/>
+      <c r="B16" s="50">
+        <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
-      <c r="C16" s="64" t="s">
-        <v>165</v>
-      </c>
-      <c r="D16" s="40" t="s">
+      <c r="C16" s="65" t="s">
+        <v>158</v>
+      </c>
+      <c r="D16" s="38" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="40" t="s">
-        <v>46</v>
-      </c>
-      <c r="F16" s="41" t="s">
-        <v>203</v>
-      </c>
-      <c r="G16" s="77" t="s">
-        <v>100</v>
-      </c>
-      <c r="H16" s="41" t="s">
-        <v>125</v>
-      </c>
-      <c r="I16" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J16" s="41" t="s">
-        <v>184</v>
-      </c>
-      <c r="K16" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L16" s="79">
+      <c r="E16" s="38" t="s">
+        <v>44</v>
+      </c>
+      <c r="F16" s="39" t="s">
+        <v>73</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>95</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>119</v>
+      </c>
+      <c r="I16" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="J16" s="39" t="s">
+        <v>177</v>
+      </c>
+      <c r="K16" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="L16" s="73">
         <v>1</v>
       </c>
-      <c r="M16" s="40">
+      <c r="M16" s="38">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N16" s="41">
+      <c r="N16" s="39">
         <v>25</v>
       </c>
-      <c r="O16" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P16" s="53">
-        <v>0.1772</v>
-      </c>
-      <c r="Q16" s="43">
-        <f t="shared" ref="Q16" si="5">P16*N16</f>
-        <v>4.43</v>
-      </c>
-      <c r="R16" s="40"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="O16" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P16" s="52">
+        <v>6.1699999999999998E-2</v>
+      </c>
+      <c r="Q16" s="42">
+        <f>P16*N16</f>
+        <v>1.5425</v>
+      </c>
+      <c r="R16" s="38"/>
+    </row>
+    <row r="17" spans="1:18" ht="36" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="50">
-        <f>ROW(B17) - ROW($B$9)</f>
+      <c r="B17" s="51">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="65" t="s">
-        <v>165</v>
-      </c>
-      <c r="D17" s="38" t="s">
+      <c r="C17" s="64" t="s">
+        <v>159</v>
+      </c>
+      <c r="D17" s="40" t="s">
         <v>15</v>
       </c>
-      <c r="E17" s="38" t="s">
-        <v>47</v>
-      </c>
-      <c r="F17" s="39" t="s">
-        <v>77</v>
-      </c>
-      <c r="G17" s="38" t="s">
-        <v>101</v>
-      </c>
-      <c r="H17" s="39" t="s">
-        <v>126</v>
-      </c>
-      <c r="I17" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J17" s="39" t="s">
-        <v>185</v>
-      </c>
-      <c r="K17" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L17" s="78">
+      <c r="E17" s="40" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="41" t="s">
+        <v>196</v>
+      </c>
+      <c r="G17" s="40" t="s">
+        <v>74</v>
+      </c>
+      <c r="H17" s="41" t="s">
+        <v>118</v>
+      </c>
+      <c r="I17" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J17" s="41" t="s">
+        <v>178</v>
+      </c>
+      <c r="K17" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="L17" s="74">
+        <v>4</v>
+      </c>
+      <c r="M17" s="40">
+        <f t="shared" si="1"/>
+        <v>80</v>
+      </c>
+      <c r="N17" s="41">
+        <v>100</v>
+      </c>
+      <c r="O17" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P17" s="53">
+        <v>2.8000000000000001E-2</v>
+      </c>
+      <c r="Q17" s="43">
+        <f t="shared" ref="Q17" si="5">P17*N17</f>
+        <v>2.8000000000000003</v>
+      </c>
+      <c r="R17" s="40"/>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="1"/>
+      <c r="B18" s="50">
+        <f>ROW(B18) - ROW($B$9)</f>
+        <v>9</v>
+      </c>
+      <c r="C18" s="63" t="s">
+        <v>160</v>
+      </c>
+      <c r="D18" s="38" t="s">
+        <v>16</v>
+      </c>
+      <c r="E18" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>195</v>
+      </c>
+      <c r="G18" s="38" t="s">
+        <v>75</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>120</v>
+      </c>
+      <c r="I18" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="J18" s="39" t="s">
+        <v>169</v>
+      </c>
+      <c r="K18" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="L18" s="73">
         <v>1</v>
       </c>
-      <c r="M17" s="38">
+      <c r="M18" s="38">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N17" s="39">
-        <v>25</v>
-      </c>
-      <c r="O17" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P17" s="52">
-        <v>6.1699999999999998E-2</v>
-      </c>
-      <c r="Q17" s="42">
-        <f>P17*N17</f>
-        <v>1.5425</v>
-      </c>
-      <c r="R17" s="38"/>
-    </row>
-    <row r="18" spans="1:18" ht="36" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="51">
+      <c r="N18" s="39">
+        <v>22</v>
+      </c>
+      <c r="O18" s="70" t="s">
+        <v>207</v>
+      </c>
+      <c r="P18" s="52">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="Q18" s="42">
+        <f>P18*N18</f>
+        <v>55.22</v>
+      </c>
+      <c r="R18" s="38"/>
+    </row>
+    <row r="19" spans="1:18" ht="24" x14ac:dyDescent="0.3">
+      <c r="A19" s="1"/>
+      <c r="B19" s="51">
         <f t="shared" si="0"/>
-        <v>9</v>
-      </c>
-      <c r="C18" s="64" t="s">
-        <v>166</v>
-      </c>
-      <c r="D18" s="40" t="s">
-        <v>16</v>
-      </c>
-      <c r="E18" s="40" t="s">
-        <v>48</v>
-      </c>
-      <c r="F18" s="41" t="s">
-        <v>204</v>
-      </c>
-      <c r="G18" s="40" t="s">
-        <v>78</v>
-      </c>
-      <c r="H18" s="41" t="s">
-        <v>124</v>
-      </c>
-      <c r="I18" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J18" s="41" t="s">
-        <v>186</v>
-      </c>
-      <c r="K18" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L18" s="79">
-        <v>4</v>
-      </c>
-      <c r="M18" s="40">
-        <f t="shared" si="1"/>
-        <v>80</v>
-      </c>
-      <c r="N18" s="41">
-        <v>100</v>
-      </c>
-      <c r="O18" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P18" s="53">
-        <v>2.8000000000000001E-2</v>
-      </c>
-      <c r="Q18" s="43">
-        <f t="shared" ref="Q18" si="6">P18*N18</f>
-        <v>2.8000000000000003</v>
-      </c>
-      <c r="R18" s="40"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="50">
-        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
-      <c r="C19" s="63" t="s">
-        <v>167</v>
-      </c>
-      <c r="D19" s="38" t="s">
+      <c r="C19" s="64" t="s">
+        <v>159</v>
+      </c>
+      <c r="D19" s="40" t="s">
         <v>17</v>
       </c>
-      <c r="E19" s="38" t="s">
-        <v>49</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>203</v>
-      </c>
-      <c r="G19" s="38" t="s">
-        <v>79</v>
-      </c>
-      <c r="H19" s="39" t="s">
-        <v>127</v>
-      </c>
-      <c r="I19" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J19" s="39" t="s">
-        <v>176</v>
-      </c>
-      <c r="K19" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L19" s="78">
+      <c r="E19" s="40" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" s="41" t="s">
+        <v>76</v>
+      </c>
+      <c r="G19" s="40" t="s">
+        <v>96</v>
+      </c>
+      <c r="H19" s="41" t="s">
+        <v>121</v>
+      </c>
+      <c r="I19" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J19" s="41" t="s">
+        <v>179</v>
+      </c>
+      <c r="K19" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="L19" s="74">
         <v>1</v>
       </c>
-      <c r="M19" s="38">
+      <c r="M19" s="40">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N19" s="39">
-        <v>22</v>
-      </c>
-      <c r="O19" s="74" t="s">
-        <v>215</v>
-      </c>
-      <c r="P19" s="52">
-        <v>2.5099999999999998</v>
-      </c>
-      <c r="Q19" s="42">
-        <f>P19*N19</f>
-        <v>55.22</v>
-      </c>
-      <c r="R19" s="38"/>
-    </row>
-    <row r="20" spans="1:18" ht="36" x14ac:dyDescent="0.25">
+      <c r="N19" s="41">
+        <v>25</v>
+      </c>
+      <c r="O19" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P19" s="53">
+        <v>8.7599999999999997E-2</v>
+      </c>
+      <c r="Q19" s="43">
+        <f t="shared" ref="Q19" si="6">P19*N19</f>
+        <v>2.19</v>
+      </c>
+      <c r="R19" s="40"/>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="51">
-        <f t="shared" si="0"/>
+      <c r="B20" s="50">
+        <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
-      <c r="C20" s="64" t="s">
-        <v>166</v>
-      </c>
-      <c r="D20" s="40" t="s">
+      <c r="C20" s="63" t="s">
+        <v>161</v>
+      </c>
+      <c r="D20" s="38" t="s">
         <v>18</v>
       </c>
-      <c r="E20" s="40" t="s">
-        <v>50</v>
-      </c>
-      <c r="F20" s="41" t="s">
-        <v>80</v>
-      </c>
-      <c r="G20" s="40" t="s">
-        <v>102</v>
-      </c>
-      <c r="H20" s="41" t="s">
-        <v>128</v>
-      </c>
-      <c r="I20" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J20" s="41" t="s">
-        <v>187</v>
-      </c>
-      <c r="K20" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L20" s="79">
+      <c r="E20" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="F20" s="39" t="s">
+        <v>77</v>
+      </c>
+      <c r="G20" s="66" t="s">
+        <v>97</v>
+      </c>
+      <c r="H20" s="39" t="s">
+        <v>122</v>
+      </c>
+      <c r="I20" s="38" t="s">
+        <v>202</v>
+      </c>
+      <c r="J20" s="39" t="s">
+        <v>180</v>
+      </c>
+      <c r="K20" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="L20" s="73">
         <v>1</v>
       </c>
-      <c r="M20" s="40">
+      <c r="M20" s="38">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N20" s="41">
-        <v>25</v>
-      </c>
-      <c r="O20" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P20" s="53">
-        <v>8.7599999999999997E-2</v>
-      </c>
-      <c r="Q20" s="43">
-        <f t="shared" ref="Q20" si="7">P20*N20</f>
-        <v>2.19</v>
-      </c>
-      <c r="R20" s="40"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="N20" s="39">
+        <v>30</v>
+      </c>
+      <c r="O20" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P20" s="52">
+        <v>3.7900000000000003E-2</v>
+      </c>
+      <c r="Q20" s="42">
+        <f>P20*N20</f>
+        <v>1.137</v>
+      </c>
+      <c r="R20" s="38"/>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="50">
-        <f>ROW(B21) - ROW($B$9)</f>
+      <c r="B21" s="51">
+        <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="63" t="s">
-        <v>168</v>
-      </c>
-      <c r="D21" s="38" t="s">
+      <c r="C21" s="64" t="s">
+        <v>162</v>
+      </c>
+      <c r="D21" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="E21" s="38" t="s">
-        <v>51</v>
-      </c>
-      <c r="F21" s="39" t="s">
-        <v>81</v>
-      </c>
-      <c r="G21" s="67" t="s">
-        <v>103</v>
-      </c>
-      <c r="H21" s="39" t="s">
-        <v>129</v>
-      </c>
-      <c r="I21" s="38" t="s">
-        <v>210</v>
-      </c>
-      <c r="J21" s="39" t="s">
-        <v>188</v>
-      </c>
-      <c r="K21" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L21" s="78">
+      <c r="E21" s="40" t="s">
+        <v>49</v>
+      </c>
+      <c r="F21" s="41" t="s">
+        <v>195</v>
+      </c>
+      <c r="G21" s="40" t="s">
+        <v>78</v>
+      </c>
+      <c r="H21" s="41" t="s">
+        <v>123</v>
+      </c>
+      <c r="I21" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J21" s="41" t="s">
+        <v>169</v>
+      </c>
+      <c r="K21" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="L21" s="74">
         <v>1</v>
       </c>
-      <c r="M21" s="38">
+      <c r="M21" s="40">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N21" s="39">
-        <v>30</v>
-      </c>
-      <c r="O21" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P21" s="52">
-        <v>3.7900000000000003E-2</v>
-      </c>
-      <c r="Q21" s="42">
-        <f>P21*N21</f>
-        <v>1.137</v>
-      </c>
-      <c r="R21" s="38"/>
-    </row>
-    <row r="22" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="N21" s="41">
+        <v>25</v>
+      </c>
+      <c r="O21" s="69" t="s">
+        <v>208</v>
+      </c>
+      <c r="P21" s="53">
+        <v>0.30840000000000001</v>
+      </c>
+      <c r="Q21" s="43">
+        <f t="shared" ref="Q21" si="7">P21*N21</f>
+        <v>7.71</v>
+      </c>
+      <c r="R21" s="40"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="51">
+      <c r="B22" s="50">
+        <f>ROW(B22) - ROW($B$9)</f>
+        <v>13</v>
+      </c>
+      <c r="C22" s="63" t="s">
+        <v>163</v>
+      </c>
+      <c r="D22" s="38" t="s">
+        <v>20</v>
+      </c>
+      <c r="E22" s="38" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="39" t="s">
+        <v>72</v>
+      </c>
+      <c r="G22" s="38" t="s">
+        <v>98</v>
+      </c>
+      <c r="H22" s="39" t="s">
+        <v>124</v>
+      </c>
+      <c r="I22" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="J22" s="39" t="s">
+        <v>181</v>
+      </c>
+      <c r="K22" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="L22" s="73">
+        <v>2</v>
+      </c>
+      <c r="M22" s="38">
+        <f t="shared" si="1"/>
+        <v>40</v>
+      </c>
+      <c r="N22" s="39">
+        <v>60</v>
+      </c>
+      <c r="O22" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P22" s="52">
+        <v>3.0599999999999999E-2</v>
+      </c>
+      <c r="Q22" s="42">
+        <f>P22*N22</f>
+        <v>1.8359999999999999</v>
+      </c>
+      <c r="R22" s="38"/>
+    </row>
+    <row r="23" spans="1:18" ht="60" x14ac:dyDescent="0.3">
+      <c r="A23" s="1"/>
+      <c r="B23" s="51">
         <f t="shared" si="0"/>
-        <v>13</v>
-      </c>
-      <c r="C22" s="64" t="s">
-        <v>169</v>
-      </c>
-      <c r="D22" s="40" t="s">
-        <v>20</v>
-      </c>
-      <c r="E22" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="64" t="s">
+        <v>164</v>
+      </c>
+      <c r="D23" s="40" t="s">
+        <v>21</v>
+      </c>
+      <c r="E23" s="40" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="G23" s="40" t="s">
+        <v>99</v>
+      </c>
+      <c r="H23" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J23" s="41" t="s">
+        <v>182</v>
+      </c>
+      <c r="K23" s="40" t="s">
+        <v>140</v>
+      </c>
+      <c r="L23" s="74">
+        <v>40</v>
+      </c>
+      <c r="M23" s="40">
+        <f t="shared" si="1"/>
+        <v>800</v>
+      </c>
+      <c r="N23" s="41">
+        <v>900</v>
+      </c>
+      <c r="O23" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P23" s="53">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="Q23" s="43">
+        <f t="shared" ref="Q23" si="8">P23*N23</f>
+        <v>0.72000000000000008</v>
+      </c>
+      <c r="R23" s="40"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" s="1"/>
+      <c r="B24" s="50">
+        <f>ROW(B24) - ROW($B$9)</f>
+        <v>15</v>
+      </c>
+      <c r="C24" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="D24" s="38" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="F22" s="41" t="s">
+      <c r="F24" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="G24" s="38" t="s">
+        <v>100</v>
+      </c>
+      <c r="H24" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="I24" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="J24" s="39" t="s">
+        <v>183</v>
+      </c>
+      <c r="K24" s="38" t="s">
+        <v>141</v>
+      </c>
+      <c r="L24" s="73">
+        <v>7</v>
+      </c>
+      <c r="M24" s="38">
+        <f t="shared" si="1"/>
+        <v>140</v>
+      </c>
+      <c r="N24" s="39">
+        <v>200</v>
+      </c>
+      <c r="O24" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P24" s="52">
+        <v>1E-3</v>
+      </c>
+      <c r="Q24" s="42">
+        <f>P24*N24</f>
+        <v>0.2</v>
+      </c>
+      <c r="R24" s="38"/>
+    </row>
+    <row r="25" spans="1:18" ht="24" x14ac:dyDescent="0.3">
+      <c r="A25" s="1"/>
+      <c r="B25" s="51">
+        <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="C25" s="64" t="s">
+        <v>164</v>
+      </c>
+      <c r="D25" s="40" t="s">
+        <v>23</v>
+      </c>
+      <c r="E25" s="40" t="s">
+        <v>53</v>
+      </c>
+      <c r="F25" s="41" t="s">
+        <v>79</v>
+      </c>
+      <c r="G25" s="71" t="s">
+        <v>101</v>
+      </c>
+      <c r="H25" s="41" t="s">
+        <v>125</v>
+      </c>
+      <c r="I25" s="40" t="s">
         <v>203</v>
       </c>
-      <c r="G22" s="40" t="s">
-        <v>82</v>
-      </c>
-      <c r="H22" s="41" t="s">
-        <v>130</v>
-      </c>
-      <c r="I22" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J22" s="41" t="s">
-        <v>176</v>
-      </c>
-      <c r="K22" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L22" s="79">
+      <c r="J25" s="41" t="s">
+        <v>184</v>
+      </c>
+      <c r="K25" s="40" t="s">
+        <v>142</v>
+      </c>
+      <c r="L25" s="74">
         <v>1</v>
       </c>
-      <c r="M22" s="40">
+      <c r="M25" s="40">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="N22" s="41">
-        <v>25</v>
-      </c>
-      <c r="O22" s="73" t="s">
-        <v>216</v>
-      </c>
-      <c r="P22" s="53">
-        <v>0.30840000000000001</v>
-      </c>
-      <c r="Q22" s="43">
-        <f t="shared" ref="Q22" si="8">P22*N22</f>
-        <v>7.71</v>
-      </c>
-      <c r="R22" s="40"/>
-    </row>
-    <row r="23" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="50">
-        <f>ROW(B23) - ROW($B$9)</f>
-        <v>14</v>
-      </c>
-      <c r="C23" s="63" t="s">
-        <v>170</v>
-      </c>
-      <c r="D23" s="38" t="s">
-        <v>21</v>
-      </c>
-      <c r="E23" s="38" t="s">
-        <v>53</v>
-      </c>
-      <c r="F23" s="39" t="s">
-        <v>76</v>
-      </c>
-      <c r="G23" s="38" t="s">
-        <v>104</v>
-      </c>
-      <c r="H23" s="39" t="s">
-        <v>131</v>
-      </c>
-      <c r="I23" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J23" s="39" t="s">
-        <v>189</v>
-      </c>
-      <c r="K23" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L23" s="78">
+      <c r="N25" s="41">
+        <v>100</v>
+      </c>
+      <c r="O25" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P25" s="53">
+        <v>1.9E-3</v>
+      </c>
+      <c r="Q25" s="43">
+        <f t="shared" ref="Q25" si="9">P25*N25</f>
+        <v>0.19</v>
+      </c>
+      <c r="R25" s="40"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="1"/>
+      <c r="B26" s="50">
+        <f>ROW(B26) - ROW($B$9)</f>
+        <v>17</v>
+      </c>
+      <c r="C26" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="D26" s="38" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" s="38" t="s">
+        <v>54</v>
+      </c>
+      <c r="F26" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="G26" s="38" t="s">
+        <v>102</v>
+      </c>
+      <c r="H26" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="J26" s="39" t="s">
+        <v>185</v>
+      </c>
+      <c r="K26" s="38" t="s">
+        <v>143</v>
+      </c>
+      <c r="L26" s="73">
         <v>2</v>
       </c>
-      <c r="M23" s="38">
+      <c r="M26" s="38">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N23" s="39">
-        <v>60</v>
-      </c>
-      <c r="O23" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P23" s="52">
-        <v>3.0599999999999999E-2</v>
-      </c>
-      <c r="Q23" s="42">
-        <f>P23*N23</f>
-        <v>1.8359999999999999</v>
-      </c>
-      <c r="R23" s="38"/>
-    </row>
-    <row r="24" spans="1:18" ht="72" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="51">
+      <c r="N26" s="39">
+        <v>100</v>
+      </c>
+      <c r="O26" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P26" s="52">
+        <v>1E-3</v>
+      </c>
+      <c r="Q26" s="42">
+        <f>P26*N26</f>
+        <v>0.1</v>
+      </c>
+      <c r="R26" s="38"/>
+    </row>
+    <row r="27" spans="1:18" ht="36" x14ac:dyDescent="0.3">
+      <c r="A27" s="1"/>
+      <c r="B27" s="51">
         <f t="shared" si="0"/>
-        <v>15</v>
-      </c>
-      <c r="C24" s="64" t="s">
-        <v>171</v>
-      </c>
-      <c r="D24" s="40" t="s">
-        <v>22</v>
-      </c>
-      <c r="E24" s="40" t="s">
-        <v>54</v>
-      </c>
-      <c r="F24" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="G24" s="40" t="s">
-        <v>105</v>
-      </c>
-      <c r="H24" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="I24" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J24" s="41" t="s">
-        <v>190</v>
-      </c>
-      <c r="K24" s="40" t="s">
-        <v>147</v>
-      </c>
-      <c r="L24" s="79">
-        <v>40</v>
-      </c>
-      <c r="M24" s="40">
-        <f t="shared" si="1"/>
-        <v>800</v>
-      </c>
-      <c r="N24" s="41">
-        <v>900</v>
-      </c>
-      <c r="O24" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P24" s="53">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="Q24" s="43">
-        <f t="shared" ref="Q24" si="9">P24*N24</f>
-        <v>0.72000000000000008</v>
-      </c>
-      <c r="R24" s="40"/>
-    </row>
-    <row r="25" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="50">
-        <f>ROW(B25) - ROW($B$9)</f>
-        <v>16</v>
-      </c>
-      <c r="C25" s="63" t="s">
-        <v>171</v>
-      </c>
-      <c r="D25" s="38" t="s">
-        <v>23</v>
-      </c>
-      <c r="E25" s="38" t="s">
+        <v>18</v>
+      </c>
+      <c r="C27" s="64" t="s">
+        <v>164</v>
+      </c>
+      <c r="D27" s="40" t="s">
+        <v>25</v>
+      </c>
+      <c r="E27" s="40" t="s">
         <v>55</v>
       </c>
-      <c r="F25" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="G25" s="38" t="s">
-        <v>106</v>
-      </c>
-      <c r="H25" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="I25" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J25" s="39" t="s">
-        <v>191</v>
-      </c>
-      <c r="K25" s="38" t="s">
-        <v>148</v>
-      </c>
-      <c r="L25" s="78">
-        <v>7</v>
-      </c>
-      <c r="M25" s="38">
-        <f t="shared" si="1"/>
-        <v>140</v>
-      </c>
-      <c r="N25" s="39">
-        <v>200</v>
-      </c>
-      <c r="O25" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P25" s="52">
-        <v>1E-3</v>
-      </c>
-      <c r="Q25" s="42">
-        <f>P25*N25</f>
-        <v>0.2</v>
-      </c>
-      <c r="R25" s="38"/>
-    </row>
-    <row r="26" spans="1:18" ht="36" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="51">
-        <f t="shared" si="0"/>
-        <v>17</v>
-      </c>
-      <c r="C26" s="64" t="s">
-        <v>171</v>
-      </c>
-      <c r="D26" s="40" t="s">
-        <v>24</v>
-      </c>
-      <c r="E26" s="40" t="s">
-        <v>56</v>
-      </c>
-      <c r="F26" s="41" t="s">
-        <v>83</v>
-      </c>
-      <c r="G26" s="76" t="s">
-        <v>107</v>
-      </c>
-      <c r="H26" s="41" t="s">
-        <v>132</v>
-      </c>
-      <c r="I26" s="40" t="s">
-        <v>211</v>
-      </c>
-      <c r="J26" s="41" t="s">
-        <v>192</v>
-      </c>
-      <c r="K26" s="40" t="s">
-        <v>149</v>
-      </c>
-      <c r="L26" s="79">
-        <v>1</v>
-      </c>
-      <c r="M26" s="40">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N26" s="41">
-        <v>100</v>
-      </c>
-      <c r="O26" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P26" s="53">
-        <v>1.9E-3</v>
-      </c>
-      <c r="Q26" s="43">
-        <f t="shared" ref="Q26" si="10">P26*N26</f>
-        <v>0.19</v>
-      </c>
-      <c r="R26" s="40"/>
-    </row>
-    <row r="27" spans="1:18" ht="24" x14ac:dyDescent="0.25">
-      <c r="A27" s="1"/>
-      <c r="B27" s="50">
-        <f>ROW(B27) - ROW($B$9)</f>
-        <v>18</v>
-      </c>
-      <c r="C27" s="63" t="s">
-        <v>171</v>
-      </c>
-      <c r="D27" s="38" t="s">
-        <v>25</v>
-      </c>
-      <c r="E27" s="38" t="s">
-        <v>57</v>
-      </c>
-      <c r="F27" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="G27" s="38" t="s">
-        <v>108</v>
-      </c>
-      <c r="H27" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="I27" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J27" s="39" t="s">
-        <v>193</v>
-      </c>
-      <c r="K27" s="38" t="s">
-        <v>150</v>
-      </c>
-      <c r="L27" s="78">
+      <c r="F27" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="G27" s="40" t="s">
+        <v>103</v>
+      </c>
+      <c r="H27" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="I27" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J27" s="41" t="s">
+        <v>186</v>
+      </c>
+      <c r="K27" s="40" t="s">
+        <v>144</v>
+      </c>
+      <c r="L27" s="74">
         <v>2</v>
       </c>
-      <c r="M27" s="38">
+      <c r="M27" s="40">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N27" s="39">
+      <c r="N27" s="41">
         <v>100</v>
       </c>
-      <c r="O27" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P27" s="52">
-        <v>1E-3</v>
-      </c>
-      <c r="Q27" s="42">
-        <f>P27*N27</f>
-        <v>0.1</v>
-      </c>
-      <c r="R27" s="38"/>
-    </row>
-    <row r="28" spans="1:18" ht="36" x14ac:dyDescent="0.25">
+      <c r="O27" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P27" s="53">
+        <v>1.2999999999999999E-3</v>
+      </c>
+      <c r="Q27" s="43">
+        <f t="shared" ref="Q27" si="10">P27*N27</f>
+        <v>0.13</v>
+      </c>
+      <c r="R27" s="40"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A28" s="1"/>
-      <c r="B28" s="51">
-        <f t="shared" si="0"/>
+      <c r="B28" s="50">
+        <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
-      <c r="C28" s="64" t="s">
-        <v>171</v>
-      </c>
-      <c r="D28" s="40" t="s">
+      <c r="C28" s="63" t="s">
+        <v>164</v>
+      </c>
+      <c r="D28" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E28" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="F28" s="41" t="s">
-        <v>84</v>
-      </c>
-      <c r="G28" s="40" t="s">
-        <v>109</v>
-      </c>
-      <c r="H28" s="41" t="s">
-        <v>123</v>
-      </c>
-      <c r="I28" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J28" s="41" t="s">
-        <v>194</v>
-      </c>
-      <c r="K28" s="40" t="s">
-        <v>151</v>
-      </c>
-      <c r="L28" s="79">
+      <c r="E28" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="F28" s="39" t="s">
+        <v>80</v>
+      </c>
+      <c r="G28" s="66" t="s">
+        <v>104</v>
+      </c>
+      <c r="H28" s="39" t="s">
+        <v>117</v>
+      </c>
+      <c r="I28" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="J28" s="39" t="s">
+        <v>187</v>
+      </c>
+      <c r="K28" s="38" t="s">
+        <v>145</v>
+      </c>
+      <c r="L28" s="73">
         <v>2</v>
       </c>
-      <c r="M28" s="40">
+      <c r="M28" s="38">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N28" s="41">
-        <v>100</v>
-      </c>
-      <c r="O28" s="73" t="s">
-        <v>214</v>
-      </c>
-      <c r="P28" s="53">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="Q28" s="43">
-        <f t="shared" ref="Q28" si="11">P28*N28</f>
-        <v>0.13</v>
-      </c>
-      <c r="R28" s="40"/>
-    </row>
-    <row r="29" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="N28" s="39">
+        <v>50</v>
+      </c>
+      <c r="O28" s="70" t="s">
+        <v>206</v>
+      </c>
+      <c r="P28" s="52">
+        <v>2.7000000000000001E-3</v>
+      </c>
+      <c r="Q28" s="42">
+        <f>P28*N28</f>
+        <v>0.13500000000000001</v>
+      </c>
+      <c r="R28" s="38"/>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A29" s="1"/>
-      <c r="B29" s="50">
-        <f>ROW(B29) - ROW($B$9)</f>
+      <c r="B29" s="51">
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="63" t="s">
-        <v>171</v>
-      </c>
-      <c r="D29" s="38" t="s">
+      <c r="C29" s="64" t="s">
+        <v>164</v>
+      </c>
+      <c r="D29" s="40" t="s">
         <v>27</v>
       </c>
-      <c r="E29" s="38" t="s">
-        <v>59</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>84</v>
-      </c>
-      <c r="G29" s="67" t="s">
-        <v>110</v>
-      </c>
-      <c r="H29" s="39" t="s">
-        <v>123</v>
-      </c>
-      <c r="I29" s="38" t="s">
-        <v>212</v>
-      </c>
-      <c r="J29" s="39" t="s">
-        <v>195</v>
-      </c>
-      <c r="K29" s="38" t="s">
-        <v>152</v>
-      </c>
-      <c r="L29" s="78">
+      <c r="E29" s="40" t="s">
+        <v>57</v>
+      </c>
+      <c r="F29" s="41" t="s">
+        <v>80</v>
+      </c>
+      <c r="G29" s="40" t="s">
+        <v>105</v>
+      </c>
+      <c r="H29" s="41" t="s">
+        <v>117</v>
+      </c>
+      <c r="I29" s="40" t="s">
+        <v>169</v>
+      </c>
+      <c r="J29" s="41" t="s">
+        <v>188</v>
+      </c>
+      <c r="K29" s="40" t="s">
+        <v>146</v>
+      </c>
+      <c r="L29" s="74">
         <v>2</v>
       </c>
-      <c r="M29" s="38">
+      <c r="M29" s="40">
         <f t="shared" si="1"/>
         <v>40</v>
       </c>
-      <c r="N29" s="39">
-        <v>50</v>
-      </c>
-      <c r="O29" s="74" t="s">
-        <v>214</v>
-      </c>
-      <c r="P29" s="52">
-        <v>2.7000000000000001E-3</v>
-      </c>
-      <c r="Q29" s="42">
-        <f>P29*N29</f>
-        <v>0.13500000000000001</v>
-      </c>
-      <c r="R29" s="38"/>
-    </row>
-    <row r="30" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="N29" s="41">
+        <v>100</v>
+      </c>
+      <c r="O29" s="69" t="s">
+        <v>206</v>
+      </c>
+      <c r="P29" s="53">
+        <v>8.9999999999999998E-4</v>
+      </c>
+      <c r="Q29" s="43">
+        <f t="shared" ref="Q29" si="11">P29*N29</f>
+        <v>0.09</v>
+      </c>
+      <c r="R29" s="40"/>
+    </row>
+    <row r="30" spans="1:18" ht="48" x14ac:dyDescent="0.3">
       <c r="A30" s="1"/>
       <c r="B30" s="51">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
       <c r="C30" s="64" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="D30" s="40" t="s">
         <v>28</v>
       </c>
       <c r="E30" s="40" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="F30" s="41" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="G30" s="40" t="s">
-        <v>111</v>
+        <v>81</v>
       </c>
       <c r="H30" s="41" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="I30" s="40" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J30" s="41" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="K30" s="40" t="s">
-        <v>153</v>
-      </c>
-      <c r="L30" s="79">
-        <v>2</v>
+        <v>169</v>
+      </c>
+      <c r="L30" s="74">
+        <v>1</v>
       </c>
       <c r="M30" s="40">
         <f t="shared" si="1"/>
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="N30" s="41">
-        <v>100</v>
-      </c>
-      <c r="O30" s="73" t="s">
-        <v>214</v>
+        <v>30</v>
+      </c>
+      <c r="O30" s="68" t="s">
+        <v>206</v>
       </c>
       <c r="P30" s="53">
-        <v>8.9999999999999998E-4</v>
+        <v>4.1399999999999999E-2</v>
       </c>
       <c r="Q30" s="43">
         <f t="shared" ref="Q30" si="12">P30*N30</f>
-        <v>0.09</v>
+        <v>1.242</v>
       </c>
       <c r="R30" s="40"/>
     </row>
-    <row r="31" spans="1:18" ht="24" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A31" s="1"/>
       <c r="B31" s="50">
         <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
-      <c r="C31" s="66" t="s">
-        <v>85</v>
-      </c>
-      <c r="D31" s="67" t="s">
+      <c r="C31" s="63" t="s">
+        <v>166</v>
+      </c>
+      <c r="D31" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="E31" s="67" t="s">
-        <v>61</v>
-      </c>
-      <c r="F31" s="68" t="s">
-        <v>176</v>
-      </c>
-      <c r="G31" s="67" t="s">
-        <v>85</v>
-      </c>
-      <c r="H31" s="68" t="s">
-        <v>176</v>
-      </c>
-      <c r="I31" s="67" t="s">
-        <v>176</v>
-      </c>
-      <c r="J31" s="68" t="s">
-        <v>176</v>
-      </c>
-      <c r="K31" s="67" t="s">
-        <v>176</v>
-      </c>
-      <c r="L31" s="80">
-        <v>8</v>
-      </c>
-      <c r="M31" s="67">
+      <c r="E31" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="F31" s="39" t="s">
+        <v>197</v>
+      </c>
+      <c r="G31" s="66" t="s">
+        <v>106</v>
+      </c>
+      <c r="H31" s="39" t="s">
+        <v>127</v>
+      </c>
+      <c r="I31" s="38" t="s">
+        <v>205</v>
+      </c>
+      <c r="J31" s="39" t="s">
+        <v>190</v>
+      </c>
+      <c r="K31" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="L31" s="73">
+        <v>1</v>
+      </c>
+      <c r="M31" s="38">
         <f t="shared" si="1"/>
-        <v>160</v>
-      </c>
-      <c r="N31" s="68">
-        <v>160</v>
-      </c>
-      <c r="O31" s="75" t="s">
-        <v>176</v>
-      </c>
-      <c r="P31" s="69" t="s">
-        <v>176</v>
-      </c>
-      <c r="Q31" s="70" t="s">
-        <v>176</v>
-      </c>
-      <c r="R31" s="67"/>
-    </row>
-    <row r="32" spans="1:18" ht="60" x14ac:dyDescent="0.25">
+        <v>20</v>
+      </c>
+      <c r="N31" s="39">
+        <v>22</v>
+      </c>
+      <c r="O31" s="67" t="s">
+        <v>206</v>
+      </c>
+      <c r="P31" s="52">
+        <v>10.652799999999999</v>
+      </c>
+      <c r="Q31" s="42">
+        <f>P31*N31</f>
+        <v>234.36159999999998</v>
+      </c>
+      <c r="R31" s="93" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A32" s="1"/>
       <c r="B32" s="51">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
       <c r="C32" s="64" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="D32" s="40" t="s">
         <v>30</v>
       </c>
       <c r="E32" s="40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F32" s="41" t="s">
-        <v>203</v>
-      </c>
-      <c r="G32" s="40" t="s">
-        <v>86</v>
+        <v>82</v>
+      </c>
+      <c r="G32" s="72" t="s">
+        <v>107</v>
       </c>
       <c r="H32" s="41" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="I32" s="40" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J32" s="41" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="K32" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L32" s="79">
+        <v>169</v>
+      </c>
+      <c r="L32" s="74">
         <v>1</v>
       </c>
       <c r="M32" s="40">
@@ -3347,54 +3292,54 @@
         <v>20</v>
       </c>
       <c r="N32" s="41">
-        <v>30</v>
-      </c>
-      <c r="O32" s="72" t="s">
-        <v>214</v>
+        <v>22</v>
+      </c>
+      <c r="O32" s="68" t="s">
+        <v>206</v>
       </c>
       <c r="P32" s="53">
-        <v>4.1399999999999999E-2</v>
+        <v>1.6387</v>
       </c>
       <c r="Q32" s="43">
         <f t="shared" ref="Q32" si="13">P32*N32</f>
-        <v>1.242</v>
+        <v>36.051400000000001</v>
       </c>
       <c r="R32" s="40"/>
     </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A33" s="1"/>
       <c r="B33" s="50">
         <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
       <c r="C33" s="63" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D33" s="38" t="s">
         <v>31</v>
       </c>
       <c r="E33" s="38" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F33" s="39" t="s">
-        <v>205</v>
-      </c>
-      <c r="G33" s="67" t="s">
-        <v>112</v>
+        <v>198</v>
+      </c>
+      <c r="G33" s="66" t="s">
+        <v>108</v>
       </c>
       <c r="H33" s="39" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="I33" s="38" t="s">
-        <v>213</v>
+        <v>108</v>
       </c>
       <c r="J33" s="39" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="K33" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L33" s="78">
+        <v>169</v>
+      </c>
+      <c r="L33" s="73">
         <v>1</v>
       </c>
       <c r="M33" s="38">
@@ -3404,54 +3349,52 @@
       <c r="N33" s="39">
         <v>22</v>
       </c>
-      <c r="O33" s="71" t="s">
-        <v>214</v>
+      <c r="O33" s="67" t="s">
+        <v>206</v>
       </c>
       <c r="P33" s="52">
-        <v>10.652799999999999</v>
+        <v>3.0720999999999998</v>
       </c>
       <c r="Q33" s="42">
         <f>P33*N33</f>
-        <v>234.36159999999998</v>
-      </c>
-      <c r="R33" s="99" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+        <v>67.586199999999991</v>
+      </c>
+      <c r="R33" s="38"/>
+    </row>
+    <row r="34" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A34" s="1"/>
       <c r="B34" s="51">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
       <c r="C34" s="64" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D34" s="40" t="s">
         <v>32</v>
       </c>
       <c r="E34" s="40" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F34" s="41" t="s">
-        <v>87</v>
-      </c>
-      <c r="G34" s="77" t="s">
-        <v>113</v>
+        <v>199</v>
+      </c>
+      <c r="G34" s="71" t="s">
+        <v>109</v>
       </c>
       <c r="H34" s="41" t="s">
-        <v>135</v>
+        <v>127</v>
       </c>
       <c r="I34" s="40" t="s">
-        <v>176</v>
+        <v>109</v>
       </c>
       <c r="J34" s="41" t="s">
-        <v>199</v>
+        <v>134</v>
       </c>
       <c r="K34" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L34" s="79">
+        <v>169</v>
+      </c>
+      <c r="L34" s="74">
         <v>1</v>
       </c>
       <c r="M34" s="40">
@@ -3461,52 +3404,52 @@
       <c r="N34" s="41">
         <v>22</v>
       </c>
-      <c r="O34" s="72" t="s">
-        <v>214</v>
+      <c r="O34" s="68" t="s">
+        <v>206</v>
       </c>
       <c r="P34" s="53">
-        <v>1.6387</v>
+        <v>1.8360000000000001</v>
       </c>
       <c r="Q34" s="43">
         <f t="shared" ref="Q34" si="14">P34*N34</f>
-        <v>36.051400000000001</v>
+        <v>40.392000000000003</v>
       </c>
       <c r="R34" s="40"/>
     </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A35" s="1"/>
       <c r="B35" s="50">
         <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="63" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D35" s="38" t="s">
         <v>33</v>
       </c>
       <c r="E35" s="38" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F35" s="39" t="s">
-        <v>206</v>
-      </c>
-      <c r="G35" s="67" t="s">
-        <v>114</v>
+        <v>83</v>
+      </c>
+      <c r="G35" s="38" t="s">
+        <v>110</v>
       </c>
       <c r="H35" s="39" t="s">
-        <v>136</v>
+        <v>128</v>
       </c>
       <c r="I35" s="38" t="s">
-        <v>114</v>
+        <v>169</v>
       </c>
       <c r="J35" s="39" t="s">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="K35" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L35" s="78">
+        <v>169</v>
+      </c>
+      <c r="L35" s="73">
         <v>1</v>
       </c>
       <c r="M35" s="38">
@@ -3514,54 +3457,54 @@
         <v>20</v>
       </c>
       <c r="N35" s="39">
-        <v>22</v>
-      </c>
-      <c r="O35" s="71" t="s">
-        <v>214</v>
+        <v>25</v>
+      </c>
+      <c r="O35" s="67" t="s">
+        <v>206</v>
       </c>
       <c r="P35" s="52">
-        <v>3.0720999999999998</v>
+        <v>0.22670000000000001</v>
       </c>
       <c r="Q35" s="42">
         <f>P35*N35</f>
-        <v>67.586199999999991</v>
+        <v>5.6675000000000004</v>
       </c>
       <c r="R35" s="38"/>
     </row>
-    <row r="36" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A36" s="1"/>
       <c r="B36" s="51">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
       <c r="C36" s="64" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D36" s="40" t="s">
-        <v>34</v>
+        <v>213</v>
       </c>
       <c r="E36" s="40" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F36" s="41" t="s">
-        <v>207</v>
-      </c>
-      <c r="G36" s="76" t="s">
-        <v>115</v>
+        <v>84</v>
+      </c>
+      <c r="G36" s="40" t="s">
+        <v>111</v>
       </c>
       <c r="H36" s="41" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="I36" s="40" t="s">
-        <v>115</v>
+        <v>169</v>
       </c>
       <c r="J36" s="41" t="s">
-        <v>141</v>
+        <v>169</v>
       </c>
       <c r="K36" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L36" s="79">
+        <v>169</v>
+      </c>
+      <c r="L36" s="74">
         <v>1</v>
       </c>
       <c r="M36" s="40">
@@ -3571,52 +3514,52 @@
       <c r="N36" s="41">
         <v>22</v>
       </c>
-      <c r="O36" s="72" t="s">
-        <v>214</v>
+      <c r="O36" s="68" t="s">
+        <v>207</v>
       </c>
       <c r="P36" s="53">
-        <v>1.8360000000000001</v>
+        <v>1.06</v>
       </c>
       <c r="Q36" s="43">
         <f t="shared" ref="Q36" si="15">P36*N36</f>
-        <v>40.392000000000003</v>
+        <v>23.32</v>
       </c>
       <c r="R36" s="40"/>
     </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A37" s="1"/>
       <c r="B37" s="50">
         <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
       <c r="C37" s="63" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D37" s="38" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E37" s="38" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F37" s="39" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="G37" s="38" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="H37" s="39" t="s">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="I37" s="38" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J37" s="39" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="K37" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="L37" s="78">
+        <v>169</v>
+      </c>
+      <c r="L37" s="73">
         <v>1</v>
       </c>
       <c r="M37" s="38">
@@ -3624,54 +3567,54 @@
         <v>20</v>
       </c>
       <c r="N37" s="39">
-        <v>25</v>
-      </c>
-      <c r="O37" s="71" t="s">
-        <v>214</v>
+        <v>22</v>
+      </c>
+      <c r="O37" s="67" t="s">
+        <v>206</v>
       </c>
       <c r="P37" s="52">
-        <v>0.22670000000000001</v>
+        <v>0.53300000000000003</v>
       </c>
       <c r="Q37" s="42">
         <f>P37*N37</f>
-        <v>5.6675000000000004</v>
+        <v>11.726000000000001</v>
       </c>
       <c r="R37" s="38"/>
     </row>
-    <row r="38" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A38" s="1"/>
       <c r="B38" s="51">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
       <c r="C38" s="64" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="D38" s="40" t="s">
-        <v>221</v>
+        <v>35</v>
       </c>
       <c r="E38" s="40" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F38" s="41" t="s">
-        <v>89</v>
+        <v>195</v>
       </c>
       <c r="G38" s="40" t="s">
-        <v>117</v>
+        <v>86</v>
       </c>
       <c r="H38" s="41" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="I38" s="40" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="J38" s="41" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="K38" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="L38" s="79">
+        <v>147</v>
+      </c>
+      <c r="L38" s="74">
         <v>1</v>
       </c>
       <c r="M38" s="40">
@@ -3681,240 +3624,130 @@
       <c r="N38" s="41">
         <v>22</v>
       </c>
-      <c r="O38" s="72" t="s">
-        <v>215</v>
+      <c r="O38" s="68" t="s">
+        <v>208</v>
       </c>
       <c r="P38" s="53">
-        <v>1.06</v>
+        <v>0.505</v>
       </c>
       <c r="Q38" s="43">
         <f t="shared" ref="Q38" si="16">P38*N38</f>
-        <v>23.32</v>
+        <v>11.11</v>
       </c>
       <c r="R38" s="40"/>
     </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1"/>
-      <c r="B39" s="50">
+      <c r="B39" s="75">
         <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
-      <c r="C39" s="63" t="s">
-        <v>173</v>
-      </c>
-      <c r="D39" s="38" t="s">
+      <c r="C39" s="76" t="s">
+        <v>167</v>
+      </c>
+      <c r="D39" s="62" t="s">
         <v>36</v>
       </c>
-      <c r="E39" s="38" t="s">
-        <v>69</v>
-      </c>
-      <c r="F39" s="39" t="s">
-        <v>90</v>
-      </c>
-      <c r="G39" s="38" t="s">
-        <v>118</v>
-      </c>
-      <c r="H39" s="39" t="s">
-        <v>126</v>
-      </c>
-      <c r="I39" s="38" t="s">
-        <v>176</v>
-      </c>
-      <c r="J39" s="39" t="s">
-        <v>202</v>
-      </c>
-      <c r="K39" s="38" t="s">
-        <v>176</v>
+      <c r="E39" s="62" t="s">
+        <v>67</v>
+      </c>
+      <c r="F39" s="77" t="s">
+        <v>195</v>
+      </c>
+      <c r="G39" s="62" t="s">
+        <v>87</v>
+      </c>
+      <c r="H39" s="77" t="s">
+        <v>132</v>
+      </c>
+      <c r="I39" s="62" t="s">
+        <v>169</v>
+      </c>
+      <c r="J39" s="77" t="s">
+        <v>169</v>
+      </c>
+      <c r="K39" s="62" t="s">
+        <v>170</v>
       </c>
       <c r="L39" s="78">
         <v>1</v>
       </c>
-      <c r="M39" s="38">
+      <c r="M39" s="62">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="N39" s="39">
         <v>22</v>
       </c>
-      <c r="O39" s="71" t="s">
-        <v>214</v>
+      <c r="O39" s="67" t="s">
+        <v>207</v>
       </c>
       <c r="P39" s="52">
-        <v>0.53300000000000003</v>
+        <v>0.69</v>
       </c>
       <c r="Q39" s="42">
         <f>P39*N39</f>
-        <v>11.726000000000001</v>
-      </c>
-      <c r="R39" s="38"/>
-    </row>
-    <row r="40" spans="1:18" x14ac:dyDescent="0.25">
+        <v>15.18</v>
+      </c>
+      <c r="R39" s="62"/>
+    </row>
+    <row r="40" spans="1:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A40" s="1"/>
-      <c r="B40" s="51">
-        <f t="shared" si="0"/>
-        <v>31</v>
-      </c>
-      <c r="C40" s="64" t="s">
-        <v>174</v>
-      </c>
-      <c r="D40" s="40" t="s">
-        <v>37</v>
-      </c>
-      <c r="E40" s="40" t="s">
-        <v>70</v>
-      </c>
-      <c r="F40" s="41" t="s">
-        <v>203</v>
-      </c>
-      <c r="G40" s="40" t="s">
-        <v>91</v>
-      </c>
-      <c r="H40" s="41" t="s">
-        <v>138</v>
-      </c>
-      <c r="I40" s="40" t="s">
-        <v>176</v>
-      </c>
-      <c r="J40" s="41" t="s">
-        <v>176</v>
-      </c>
-      <c r="K40" s="40" t="s">
-        <v>154</v>
-      </c>
-      <c r="L40" s="79">
-        <v>1</v>
-      </c>
-      <c r="M40" s="40">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N40" s="41">
-        <v>22</v>
-      </c>
-      <c r="O40" s="72" t="s">
-        <v>216</v>
-      </c>
-      <c r="P40" s="53">
-        <v>0.505</v>
-      </c>
-      <c r="Q40" s="43">
-        <f t="shared" ref="Q40" si="17">P40*N40</f>
-        <v>11.11</v>
-      </c>
-      <c r="R40" s="40"/>
-    </row>
-    <row r="41" spans="1:18" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="44"/>
+      <c r="C40" s="45"/>
+      <c r="D40" s="46"/>
+      <c r="E40" s="47"/>
+      <c r="F40" s="48"/>
+      <c r="G40" s="49"/>
+      <c r="H40" s="48"/>
+      <c r="I40" s="49"/>
+      <c r="J40" s="48"/>
+      <c r="K40" s="49"/>
+      <c r="L40" s="49"/>
+      <c r="M40" s="49"/>
+      <c r="N40" s="100" t="s">
+        <v>5</v>
+      </c>
+      <c r="O40" s="101"/>
+      <c r="P40" s="101"/>
+      <c r="Q40" s="54">
+        <f>SUM(Q10:Q39)</f>
+        <v>527.16819999999996</v>
+      </c>
+      <c r="R40" s="98"/>
+    </row>
+    <row r="41" spans="1:18" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A41" s="1"/>
-      <c r="B41" s="81">
-        <f>ROW(B41) - ROW($B$9)</f>
-        <v>32</v>
-      </c>
-      <c r="C41" s="82" t="s">
-        <v>174</v>
-      </c>
-      <c r="D41" s="62" t="s">
-        <v>38</v>
-      </c>
-      <c r="E41" s="62" t="s">
-        <v>71</v>
-      </c>
-      <c r="F41" s="83" t="s">
-        <v>203</v>
-      </c>
-      <c r="G41" s="62" t="s">
-        <v>92</v>
-      </c>
-      <c r="H41" s="83" t="s">
-        <v>139</v>
-      </c>
-      <c r="I41" s="62" t="s">
-        <v>176</v>
-      </c>
-      <c r="J41" s="83" t="s">
-        <v>176</v>
-      </c>
-      <c r="K41" s="62" t="s">
-        <v>177</v>
-      </c>
-      <c r="L41" s="84">
-        <v>1</v>
-      </c>
-      <c r="M41" s="62">
-        <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-      <c r="N41" s="39">
-        <v>22</v>
-      </c>
-      <c r="O41" s="71" t="s">
-        <v>215</v>
-      </c>
-      <c r="P41" s="52">
-        <v>0.69</v>
-      </c>
-      <c r="Q41" s="42">
-        <f>P41*N41</f>
-        <v>15.18</v>
-      </c>
-      <c r="R41" s="62"/>
-    </row>
-    <row r="42" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="1"/>
-      <c r="B42" s="44"/>
-      <c r="C42" s="45"/>
-      <c r="D42" s="46"/>
-      <c r="E42" s="47"/>
-      <c r="F42" s="48"/>
-      <c r="G42" s="49"/>
-      <c r="H42" s="48"/>
-      <c r="I42" s="49"/>
-      <c r="J42" s="48"/>
-      <c r="K42" s="49"/>
-      <c r="L42" s="49"/>
-      <c r="M42" s="49"/>
-      <c r="N42" s="106" t="s">
-        <v>5</v>
-      </c>
-      <c r="O42" s="107"/>
-      <c r="P42" s="107"/>
-      <c r="Q42" s="54">
-        <f>SUM(Q10:Q41)</f>
-        <v>531.59819999999991</v>
-      </c>
-      <c r="R42" s="104"/>
-    </row>
-    <row r="43" spans="1:18" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="1"/>
-      <c r="B43" s="25"/>
-      <c r="C43" s="37"/>
-      <c r="D43" s="9"/>
-      <c r="E43" s="10"/>
-      <c r="F43" s="10"/>
-      <c r="G43" s="10"/>
-      <c r="H43" s="10"/>
-      <c r="I43" s="10"/>
-      <c r="J43" s="10"/>
-      <c r="K43" s="10"/>
-      <c r="L43" s="10"/>
-      <c r="M43" s="10"/>
-      <c r="N43" s="106" t="s">
+      <c r="B41" s="25"/>
+      <c r="C41" s="37"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="10"/>
+      <c r="J41" s="10"/>
+      <c r="K41" s="10"/>
+      <c r="L41" s="10"/>
+      <c r="M41" s="10"/>
+      <c r="N41" s="100" t="s">
         <v>6</v>
       </c>
-      <c r="O43" s="107"/>
-      <c r="P43" s="107"/>
-      <c r="Q43" s="55">
-        <f>Q42/20</f>
-        <v>26.579909999999995</v>
-      </c>
-      <c r="R43" s="105"/>
+      <c r="O41" s="101"/>
+      <c r="P41" s="101"/>
+      <c r="Q41" s="55">
+        <f>Q40/20</f>
+        <v>26.358409999999999</v>
+      </c>
+      <c r="R41" s="99"/>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="K1:R1"/>
     <mergeCell ref="R3:R8"/>
-    <mergeCell ref="R42:R43"/>
-    <mergeCell ref="N42:P42"/>
-    <mergeCell ref="N43:P43"/>
+    <mergeCell ref="R40:R41"/>
+    <mergeCell ref="N40:P40"/>
+    <mergeCell ref="N41:P41"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="O10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
@@ -3923,34 +3756,33 @@
     <hyperlink ref="O13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
     <hyperlink ref="O14" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
     <hyperlink ref="O15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="O16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="O17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="O18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="O19" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="O20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="O21" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="O22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="O23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="O24" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="O25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="O26" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="O27" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="O28" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="O29" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="O32" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="O33" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="O34" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="O35" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="O36" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="O37" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="O39" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="O41" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="O30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="O38" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="O40" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="O16" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="O17" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="O18" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="O19" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="O20" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="O21" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="O22" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="O23" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="O24" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="O25" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="O26" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="O27" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="O28" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="O30" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="O31" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="O32" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="O33" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="O34" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="O35" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="O37" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="O39" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="O29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="O36" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="O38" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId32"/>
-  <drawing r:id="rId33"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId31"/>
+  <drawing r:id="rId32"/>
 </worksheet>
 </file>
</xml_diff>